<commit_message>
Update inventory data 2026-07-06 14:37
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{90711ED1-1A89-4CB8-846C-FB7B0586ECA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE7A84A-0225-4708-9420-D5338E202062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1395" yWindow="1290" windowWidth="16350" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="95">
   <si>
     <t>分類</t>
   </si>
@@ -359,6 +359,10 @@
   </si>
   <si>
     <t>5/13下單103卷，7/15淋膜，7/22送台北10箱，剩下7/23送台南16箱</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>6/23已完工320卷，剩餘32卷未完工，尚未入庫欣凱倉</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1547,7 +1551,9 @@
       </c>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
-      <c r="R19" s="2"/>
+      <c r="R19" s="2" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="20" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">

</xml_diff>

<commit_message>
Update inventory data 2026-07-07 14:11
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCE7A84A-0225-4708-9420-D5338E202062}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1218ECD-7B80-482A-9CBB-A983AB5BC30D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1395" yWindow="1290" windowWidth="16350" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -362,7 +362,7 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>6/23已完工320卷，剩餘32卷未完工，尚未入庫欣凱倉</t>
+    <t>6/23已完工320卷，剩餘32卷未完工</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1607,9 +1607,7 @@
       </c>
       <c r="F21" s="4"/>
       <c r="G21" s="4"/>
-      <c r="H21" s="4">
-        <v>20</v>
-      </c>
+      <c r="H21" s="4"/>
       <c r="I21" s="4"/>
       <c r="J21" s="4"/>
       <c r="K21" s="4"/>
@@ -1617,7 +1615,9 @@
       <c r="M21" s="4"/>
       <c r="N21" s="4"/>
       <c r="O21" s="4"/>
-      <c r="P21" s="4"/>
+      <c r="P21" s="4">
+        <v>20</v>
+      </c>
       <c r="Q21" s="4"/>
       <c r="R21" s="2"/>
     </row>

</xml_diff>

<commit_message>
Update inventory data 2026-07-08 10:11
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1218ECD-7B80-482A-9CBB-A983AB5BC30D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DFD6A3C-4D17-4462-BA49-0F5168FBBDEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1395" yWindow="1290" windowWidth="16350" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="184" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="98">
   <si>
     <t>分類</t>
   </si>
@@ -358,11 +358,23 @@
     <t>第一版只提示狀態，不建議採購數量，避免忽略廠商基本量與倉庫空間。</t>
   </si>
   <si>
-    <t>5/13下單103卷，7/15淋膜，7/22送台北10箱，剩下7/23送台南16箱</t>
+    <t>7/8採購40卷到臺南倉，暫定7/23台南專車</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>6/23已完工320卷，剩餘32卷未完工</t>
+    <t>7/8採購80卷到臺南倉，暫定7/23台南專車</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>7/8採購360卷到臺南倉，暫定8/13台南專車</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>5/13下單103卷，7/22送台北10箱，剩下7/23送台南16箱</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>7/8採購96卷，送台中倉，交期未知</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1067,7 +1079,7 @@
       <c r="Q5" s="4"/>
       <c r="R5" s="2"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -1099,9 +1111,11 @@
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
-      <c r="R6" s="2"/>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R6" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -1133,9 +1147,11 @@
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
-      <c r="R7" s="2"/>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R7" s="2" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="8" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
@@ -1171,9 +1187,11 @@
       <c r="O8" s="4"/>
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
-      <c r="R8" s="2"/>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R8" s="2" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="9" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
@@ -1205,9 +1223,11 @@
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
-      <c r="R9" s="2"/>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="R9" s="2" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="10" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -1239,7 +1259,9 @@
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
-      <c r="R10" s="2"/>
+      <c r="R10" s="2" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="11" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -1448,7 +1470,7 @@
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1517,7 +1539,9 @@
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
-      <c r="R18" s="2"/>
+      <c r="R18" s="2" t="s">
+        <v>97</v>
+      </c>
     </row>
     <row r="19" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
@@ -1551,9 +1575,7 @@
       </c>
       <c r="P19" s="4"/>
       <c r="Q19" s="4"/>
-      <c r="R19" s="2" t="s">
-        <v>94</v>
-      </c>
+      <c r="R19" s="2"/>
     </row>
     <row r="20" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">

</xml_diff>

<commit_message>
Update inventory data 2026-07-13 10:00
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DFD6A3C-4D17-4462-BA49-0F5168FBBDEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0526CBF0-E007-44DD-ABCC-FD52974EB51B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1395" yWindow="1290" windowWidth="16350" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="99">
   <si>
     <t>分類</t>
   </si>
@@ -375,6 +375,10 @@
   </si>
   <si>
     <t>7/8採購96卷，送台中倉，交期未知</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>7/8台北下單53卷，送北倉，交期未知</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1500,12 +1504,14 @@
       <c r="N17" s="4"/>
       <c r="O17" s="4"/>
       <c r="P17" s="4">
-        <v>16</v>
+        <v>40</v>
       </c>
       <c r="Q17" s="4">
-        <v>8</v>
-      </c>
-      <c r="R17" s="2"/>
+        <v>20</v>
+      </c>
+      <c r="R17" s="2" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="18" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">

</xml_diff>

<commit_message>
Update inventory data 2026-07-17 10:21
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0526CBF0-E007-44DD-ABCC-FD52974EB51B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD5F36C1-2F7A-4107-B87F-30FEDBF813FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1395" yWindow="1290" windowWidth="16350" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="9630" yWindow="855" windowWidth="24000" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -358,27 +358,27 @@
     <t>第一版只提示狀態，不建議採購數量，避免忽略廠商基本量與倉庫空間。</t>
   </si>
   <si>
-    <t>7/8採購40卷到臺南倉，暫定7/23台南專車</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>7/8採購80卷到臺南倉，暫定7/23台南專車</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>7/8採購360卷到臺南倉，暫定8/13台南專車</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>5/13下單103卷，7/22送台北10箱，剩下7/23送台南16箱</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>7/8採購96卷，送台中倉，交期未知</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
     <t>7/8台北下單53卷，送北倉，交期未知</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>7/8採購40卷到臺南倉，安排7/23台南專車</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>7/8採購80卷到臺南倉，安排7/23台南專車</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>5/13下單103卷，7/22送台北40卷，7/23送台南60.8卷</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1116,7 +1116,7 @@
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
       <c r="R6" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="7" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
@@ -1152,7 +1152,7 @@
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
       <c r="R7" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="8" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
@@ -1192,7 +1192,7 @@
       <c r="P8" s="4"/>
       <c r="Q8" s="4"/>
       <c r="R8" s="2" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="9" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
@@ -1228,7 +1228,7 @@
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
       <c r="R9" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
@@ -1264,7 +1264,7 @@
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
       <c r="R10" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1474,7 +1474,7 @@
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
       <c r="R16" s="2" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
     </row>
     <row r="17" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1510,7 +1510,7 @@
         <v>20</v>
       </c>
       <c r="R17" s="2" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
     </row>
     <row r="18" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -1546,7 +1546,7 @@
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
       <c r="R18" s="2" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
     </row>
     <row r="19" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Update inventory data 2026-07-24 12:57
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD5F36C1-2F7A-4107-B87F-30FEDBF813FB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{866449BE-4D8C-40DF-B6C3-D77C75D1B73D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9630" yWindow="855" windowWidth="24000" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="1455" windowWidth="24000" windowHeight="14145" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="96">
   <si>
     <t>分類</t>
   </si>
@@ -367,18 +367,6 @@
   </si>
   <si>
     <t>7/8台北下單53卷，送北倉，交期未知</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>7/8採購40卷到臺南倉，安排7/23台南專車</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>7/8採購80卷到臺南倉，安排7/23台南專車</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>5/13下單103卷，7/22送台北40卷，7/23送台南60.8卷</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1083,7 +1071,7 @@
       <c r="Q5" s="4"/>
       <c r="R5" s="2"/>
     </row>
-    <row r="6" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>18</v>
       </c>
@@ -1115,11 +1103,9 @@
       <c r="O6" s="4"/>
       <c r="P6" s="4"/>
       <c r="Q6" s="4"/>
-      <c r="R6" s="2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="7" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="R6" s="2"/>
+    </row>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>18</v>
       </c>
@@ -1151,9 +1137,7 @@
       <c r="O7" s="4"/>
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
-      <c r="R7" s="2" t="s">
-        <v>96</v>
-      </c>
+      <c r="R7" s="2"/>
     </row>
     <row r="8" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
@@ -1195,7 +1179,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>18</v>
       </c>
@@ -1227,11 +1211,9 @@
       <c r="O9" s="4"/>
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
-      <c r="R9" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="10" spans="1:18" ht="31.5" x14ac:dyDescent="0.25">
+      <c r="R9" s="2"/>
+    </row>
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>18</v>
       </c>
@@ -1263,9 +1245,7 @@
       <c r="O10" s="4"/>
       <c r="P10" s="4"/>
       <c r="Q10" s="4"/>
-      <c r="R10" s="2" t="s">
-        <v>96</v>
-      </c>
+      <c r="R10" s="2"/>
     </row>
     <row r="11" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
@@ -1473,9 +1453,7 @@
       <c r="O16" s="4"/>
       <c r="P16" s="4"/>
       <c r="Q16" s="4"/>
-      <c r="R16" s="2" t="s">
-        <v>98</v>
-      </c>
+      <c r="R16" s="2"/>
     </row>
     <row r="17" spans="1:18" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">

</xml_diff>

<commit_message>
Update inventory data 2026-07-24 15:18
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3B4317D-81E0-40ED-8FDD-A32FDEB41F5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C4E4240-4402-4CD8-8DE3-5D527E58EAE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="810" windowWidth="10860" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4110" yWindow="810" windowWidth="24000" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -34,6 +34,8 @@
             <sz val="11"/>
             <color theme="1"/>
             <rFont val="新細明體"/>
+            <family val="1"/>
+            <charset val="136"/>
           </rPr>
           <t>觀察線：低於此數量列入觀察中。</t>
         </r>
@@ -46,6 +48,8 @@
             <sz val="11"/>
             <color theme="1"/>
             <rFont val="新細明體"/>
+            <family val="1"/>
+            <charset val="136"/>
           </rPr>
           <t>採購線：低於此數量列入需採購。採購線通常小於或等於觀察線。</t>
         </r>
@@ -58,6 +62,8 @@
             <sz val="11"/>
             <color theme="1"/>
             <rFont val="新細明體"/>
+            <family val="1"/>
+            <charset val="136"/>
           </rPr>
           <t>合計欄位是選填；分倉警示仍會各自判斷。</t>
         </r>
@@ -368,7 +374,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -386,6 +392,13 @@
       <sz val="9"/>
       <name val="細明體"/>
       <family val="3"/>
+      <charset val="136"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="新細明體"/>
+      <family val="1"/>
       <charset val="136"/>
     </font>
   </fonts>
@@ -655,6 +668,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AFFB71B-8257-5180-EF1A-0C7EDDED07AE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9525000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1205,12 +1272,8 @@
       <c r="E8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="4">
-        <v>100</v>
-      </c>
-      <c r="G8" s="4">
-        <v>60</v>
-      </c>
+      <c r="F8" s="4"/>
+      <c r="G8" s="4"/>
       <c r="H8" s="4"/>
       <c r="I8" s="4"/>
       <c r="J8" s="4">
@@ -1223,8 +1286,12 @@
       <c r="M8" s="4"/>
       <c r="N8" s="4"/>
       <c r="O8" s="4"/>
-      <c r="P8" s="4"/>
-      <c r="Q8" s="4"/>
+      <c r="P8" s="4">
+        <v>120</v>
+      </c>
+      <c r="Q8" s="4">
+        <v>80</v>
+      </c>
       <c r="R8" s="9" t="s">
         <v>30</v>
       </c>

</xml_diff>

<commit_message>
Update inventory data 2026-07-31 11:25
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C4E4240-4402-4CD8-8DE3-5D527E58EAE3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6E64641-3F72-4316-B220-06D133A923B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4110" yWindow="810" windowWidth="24000" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2355" yWindow="570" windowWidth="24000" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -208,9 +208,6 @@
     <t>公版PP-特殊透明,180*500</t>
   </si>
   <si>
-    <t>7/8採購96卷，送台中倉，交期未知</t>
-  </si>
-  <si>
     <t>公版PP-透明,225*500</t>
   </si>
   <si>
@@ -368,6 +365,10 @@
   </si>
   <si>
     <t>選填；填入整數時網頁顯示牌價，留白時不顯示。修改後執行一鍵更新即可更新網站。</t>
+  </si>
+  <si>
+    <t>7/8採購96卷，預計8/13送台中倉</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -475,7 +476,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -507,6 +508,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -687,6 +691,60 @@
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
               <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7AFFB71B-8257-5180-EF1A-0C7EDDED07AE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9525000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="3" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D16B7EBE-85B7-FF15-98F6-A3EC9EA9EECE}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1019,7 +1077,7 @@
         <v>17</v>
       </c>
       <c r="S1" s="10" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:19" x14ac:dyDescent="0.25">
@@ -1670,8 +1728,8 @@
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
-      <c r="R18" s="9" t="s">
-        <v>44</v>
+      <c r="R18" s="12" t="s">
+        <v>97</v>
       </c>
       <c r="S18" s="11">
         <v>1200</v>
@@ -1685,7 +1743,7 @@
         <v>28</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D19" s="3">
         <v>225</v>
@@ -1717,10 +1775,10 @@
         <v>33</v>
       </c>
       <c r="B20" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>46</v>
-      </c>
-      <c r="C20" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="D20" s="3">
         <v>180</v>
@@ -1752,10 +1810,10 @@
         <v>33</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D21" s="3">
         <v>180</v>
@@ -1785,10 +1843,10 @@
         <v>33</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D22" s="3">
         <v>130</v>
@@ -1818,10 +1876,10 @@
         <v>33</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D23" s="3">
         <v>180</v>
@@ -1851,10 +1909,10 @@
         <v>33</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D24" s="3">
         <v>130</v>
@@ -1882,10 +1940,10 @@
         <v>33</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D25" s="3">
         <v>130</v>
@@ -1914,13 +1972,13 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="C26" s="2" t="s">
         <v>54</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="D26" s="3">
         <v>130</v>
@@ -1951,13 +2009,13 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B27" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="C27" s="2" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D27" s="3">
         <v>130</v>
@@ -1984,13 +2042,13 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B28" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="C28" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D28" s="3">
         <v>130</v>
@@ -2017,13 +2075,13 @@
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B29" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B29" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="C29" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D29" s="3">
         <v>130</v>
@@ -2050,13 +2108,13 @@
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="B30" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>54</v>
-      </c>
       <c r="C30" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D30" s="3">
         <v>130</v>
@@ -2087,13 +2145,13 @@
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B31" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>60</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="D31" s="3">
         <v>130</v>
@@ -2124,13 +2182,13 @@
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D32" s="3">
         <v>130</v>
@@ -2157,13 +2215,13 @@
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D33" s="3">
         <v>130</v>
@@ -2190,13 +2248,13 @@
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D34" s="3">
         <v>130</v>
@@ -2313,18 +2371,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>65</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>67</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -2332,63 +2390,63 @@
         <v>4</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>70</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>72</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
+        <v>73</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>74</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>75</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>76</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="B8" s="6" t="s">
         <v>78</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="B9" s="6" t="s">
         <v>80</v>
-      </c>
-      <c r="B9" s="6" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>95</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>96</v>
-      </c>
-      <c r="B10" s="7" t="s">
-        <v>97</v>
       </c>
     </row>
   </sheetData>
@@ -2408,58 +2466,58 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="5" t="s">
         <v>82</v>
-      </c>
-      <c r="B1" s="5" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>84</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>86</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>88</v>
-      </c>
-      <c r="B4" s="6" t="s">
-        <v>89</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="B5" s="6" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="B6" s="6" t="s">
         <v>92</v>
-      </c>
-      <c r="B6" s="6" t="s">
-        <v>93</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="B7" s="6" t="s">
         <v>94</v>
-      </c>
-      <c r="B7" s="6" t="s">
-        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update inventory data 2026-08-11 13:09
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6E64641-3F72-4316-B220-06D133A923B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B273AD4-092F-48FD-9E1D-5EB1CDEB09BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2355" yWindow="570" windowWidth="24000" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="99">
   <si>
     <t>分類</t>
   </si>
@@ -368,6 +368,10 @@
   </si>
   <si>
     <t>7/8採購96卷，預計8/13送台中倉</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>8/10採購360卷到台中倉，交期未知</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -780,6 +784,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="4" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{436F27D8-7FE9-6FF5-0BCB-526DA744418A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9525000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1080,7 +1138,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
@@ -1116,7 +1174,9 @@
       <c r="Q2" s="4">
         <v>150</v>
       </c>
-      <c r="R2" s="9"/>
+      <c r="R2" s="12" t="s">
+        <v>98</v>
+      </c>
       <c r="S2" s="11">
         <v>600</v>
       </c>

</xml_diff>

<commit_message>
Update inventory data 2026-08-17 09:17
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B273AD4-092F-48FD-9E1D-5EB1CDEB09BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4E3EE53-1F41-44EE-ACC3-86F9C0497CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2355" yWindow="570" windowWidth="24000" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="95">
   <si>
     <t>分類</t>
   </si>
@@ -166,9 +166,6 @@
     <t>公版PP-透明,130*450</t>
   </si>
   <si>
-    <t>7/8採購360卷到臺南倉，暫定8/13台南專車</t>
-  </si>
-  <si>
     <t>公版PP-透明,160*500</t>
   </si>
   <si>
@@ -202,9 +199,6 @@
     <t>私版GPE-特殊透明,180*450</t>
   </si>
   <si>
-    <t>7/8台北下單53卷，送北倉，交期未知</t>
-  </si>
-  <si>
     <t>公版PP-特殊透明,180*500</t>
   </si>
   <si>
@@ -365,14 +359,6 @@
   </si>
   <si>
     <t>選填；填入整數時網頁顯示牌價，留白時不顯示。修改後執行一鍵更新即可更新網站。</t>
-  </si>
-  <si>
-    <t>7/8採購96卷，預計8/13送台中倉</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>8/10採購360卷到台中倉，交期未知</t>
-    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -838,6 +824,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="5" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DCCA2965-F9B6-6C3D-6727-DBC80CC59E93}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9725025"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1135,10 +1175,10 @@
         <v>17</v>
       </c>
       <c r="S1" s="10" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="2" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="2" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>18</v>
       </c>
@@ -1174,9 +1214,7 @@
       <c r="Q2" s="4">
         <v>150</v>
       </c>
-      <c r="R2" s="12" t="s">
-        <v>98</v>
-      </c>
+      <c r="R2" s="12"/>
       <c r="S2" s="11">
         <v>600</v>
       </c>
@@ -1374,7 +1412,7 @@
         <v>1200</v>
       </c>
     </row>
-    <row r="8" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>18</v>
       </c>
@@ -1410,9 +1448,7 @@
       <c r="Q8" s="4">
         <v>80</v>
       </c>
-      <c r="R8" s="9" t="s">
-        <v>30</v>
-      </c>
+      <c r="R8" s="9"/>
       <c r="S8" s="11">
         <v>600</v>
       </c>
@@ -1425,7 +1461,7 @@
         <v>28</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D9" s="3">
         <v>160</v>
@@ -1462,7 +1498,7 @@
         <v>28</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D10" s="3">
         <v>180</v>
@@ -1493,13 +1529,13 @@
     </row>
     <row r="11" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="C11" s="2" t="s">
         <v>34</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>35</v>
       </c>
       <c r="D11" s="3">
         <v>130</v>
@@ -1530,13 +1566,13 @@
     </row>
     <row r="12" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B12" s="2" t="s">
-        <v>34</v>
-      </c>
       <c r="C12" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D12" s="3">
         <v>160</v>
@@ -1567,13 +1603,13 @@
     </row>
     <row r="13" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="2" t="s">
-        <v>34</v>
-      </c>
       <c r="C13" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="D13" s="3">
         <v>130</v>
@@ -1602,13 +1638,13 @@
     </row>
     <row r="14" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D14" s="3">
         <v>130</v>
@@ -1643,13 +1679,13 @@
     </row>
     <row r="15" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D15" s="3">
         <v>130</v>
@@ -1682,13 +1718,13 @@
     </row>
     <row r="16" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D16" s="3">
         <v>225</v>
@@ -1719,13 +1755,13 @@
     </row>
     <row r="17" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D17" s="3">
         <v>180</v>
@@ -1749,22 +1785,20 @@
       <c r="Q17" s="4">
         <v>20</v>
       </c>
-      <c r="R17" s="9" t="s">
-        <v>42</v>
-      </c>
+      <c r="R17" s="9"/>
       <c r="S17" s="11">
         <v>1200</v>
       </c>
     </row>
     <row r="18" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D18" s="3">
         <v>180</v>
@@ -1788,22 +1822,20 @@
       <c r="O18" s="4"/>
       <c r="P18" s="4"/>
       <c r="Q18" s="4"/>
-      <c r="R18" s="12" t="s">
-        <v>97</v>
-      </c>
+      <c r="R18" s="12"/>
       <c r="S18" s="11">
         <v>1200</v>
       </c>
     </row>
     <row r="19" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>28</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D19" s="3">
         <v>225</v>
@@ -1832,13 +1864,13 @@
     </row>
     <row r="20" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D20" s="3">
         <v>180</v>
@@ -1867,13 +1899,13 @@
     </row>
     <row r="21" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B21" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>45</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>47</v>
       </c>
       <c r="D21" s="3">
         <v>180</v>
@@ -1900,13 +1932,13 @@
     </row>
     <row r="22" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D22" s="3">
         <v>130</v>
@@ -1933,13 +1965,13 @@
     </row>
     <row r="23" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D23" s="3">
         <v>180</v>
@@ -1966,13 +1998,13 @@
     </row>
     <row r="24" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D24" s="3">
         <v>130</v>
@@ -1997,13 +2029,13 @@
     </row>
     <row r="25" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D25" s="3">
         <v>130</v>
@@ -2032,13 +2064,13 @@
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>52</v>
-      </c>
-      <c r="B26" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="C26" s="2" t="s">
-        <v>54</v>
       </c>
       <c r="D26" s="3">
         <v>130</v>
@@ -2069,13 +2101,13 @@
     </row>
     <row r="27" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B27" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>53</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>55</v>
       </c>
       <c r="D27" s="3">
         <v>130</v>
@@ -2102,13 +2134,13 @@
     </row>
     <row r="28" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D28" s="3">
         <v>130</v>
@@ -2135,13 +2167,13 @@
     </row>
     <row r="29" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D29" s="3">
         <v>130</v>
@@ -2168,13 +2200,13 @@
     </row>
     <row r="30" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D30" s="3">
         <v>130</v>
@@ -2205,13 +2237,13 @@
     </row>
     <row r="31" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D31" s="3">
         <v>130</v>
@@ -2242,13 +2274,13 @@
     </row>
     <row r="32" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A32" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B32" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>59</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>61</v>
       </c>
       <c r="D32" s="3">
         <v>130</v>
@@ -2275,13 +2307,13 @@
     </row>
     <row r="33" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A33" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D33" s="3">
         <v>130</v>
@@ -2308,13 +2340,13 @@
     </row>
     <row r="34" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A34" s="2" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D34" s="3">
         <v>130</v>
@@ -2431,18 +2463,18 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
@@ -2450,63 +2482,63 @@
         <v>4</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="32.1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -2526,58 +2558,58 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B1" s="5" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update inventory data 2026-08-21 11:16
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4E3EE53-1F41-44EE-ACC3-86F9C0497CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA38DFB-0880-4E63-838E-204C763F47E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2355" yWindow="570" windowWidth="24000" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5805" yWindow="810" windowWidth="15465" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="97">
   <si>
     <t>分類</t>
   </si>
@@ -359,6 +359,14 @@
   </si>
   <si>
     <t>選填；填入整數時網頁顯示牌價，留白時不顯示。修改後執行一鍵更新即可更新網站。</t>
+  </si>
+  <si>
+    <t>8/17採購617卷，預計九月底完成</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>已採360卷，預計8/27(四)送台南</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -878,6 +886,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="6" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E1171977-F854-4CC2-AA24-CBFBBA32EF82}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9324975"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1297,7 +1359,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -1333,7 +1395,9 @@
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
-      <c r="R5" s="9"/>
+      <c r="R5" s="12" t="s">
+        <v>96</v>
+      </c>
       <c r="S5" s="11">
         <v>600</v>
       </c>
@@ -1559,7 +1623,9 @@
       <c r="O11" s="4"/>
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
-      <c r="R11" s="9"/>
+      <c r="R11" s="12" t="s">
+        <v>95</v>
+      </c>
       <c r="S11" s="11">
         <v>990</v>
       </c>

</xml_diff>

<commit_message>
Update inventory data 2026-08-31 09:19
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BA38DFB-0880-4E63-838E-204C763F47E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82A1535E-1E2D-4D35-A177-C5DE44011AA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5805" yWindow="810" windowWidth="15465" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2475" yWindow="810" windowWidth="25005" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="96">
   <si>
     <t>分類</t>
   </si>
@@ -362,10 +362,6 @@
   </si>
   <si>
     <t>8/17採購617卷，預計九月底完成</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>已採360卷，預計8/27(四)送台南</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -940,6 +936,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="7" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6A24DC0A-EBF2-342C-47A3-AD9913333C58}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9525000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1359,7 +1409,7 @@
         <v>540</v>
       </c>
     </row>
-    <row r="5" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>18</v>
       </c>
@@ -1395,9 +1445,7 @@
       <c r="O5" s="4"/>
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
-      <c r="R5" s="12" t="s">
-        <v>96</v>
-      </c>
+      <c r="R5" s="12"/>
       <c r="S5" s="11">
         <v>600</v>
       </c>
@@ -1621,8 +1669,12 @@
       <c r="M11" s="4"/>
       <c r="N11" s="4"/>
       <c r="O11" s="4"/>
-      <c r="P11" s="4"/>
-      <c r="Q11" s="4"/>
+      <c r="P11" s="4">
+        <v>150</v>
+      </c>
+      <c r="Q11" s="4">
+        <v>120</v>
+      </c>
       <c r="R11" s="12" t="s">
         <v>95</v>
       </c>
@@ -1719,13 +1771,9 @@
         <v>21</v>
       </c>
       <c r="F14" s="4"/>
-      <c r="G14" s="4">
-        <v>10</v>
-      </c>
+      <c r="G14" s="4"/>
       <c r="H14" s="4"/>
-      <c r="I14" s="4">
-        <v>10</v>
-      </c>
+      <c r="I14" s="4"/>
       <c r="J14" s="4">
         <v>100</v>
       </c>
@@ -1761,9 +1809,7 @@
       </c>
       <c r="F15" s="4"/>
       <c r="G15" s="4"/>
-      <c r="H15" s="4">
-        <v>30</v>
-      </c>
+      <c r="H15" s="4"/>
       <c r="I15" s="4"/>
       <c r="J15" s="4">
         <v>30</v>
@@ -1876,18 +1922,18 @@
       <c r="G18" s="4"/>
       <c r="H18" s="4"/>
       <c r="I18" s="4"/>
-      <c r="J18" s="4">
-        <v>40</v>
-      </c>
-      <c r="K18" s="4">
-        <v>28</v>
-      </c>
+      <c r="J18" s="4"/>
+      <c r="K18" s="4"/>
       <c r="L18" s="4"/>
       <c r="M18" s="4"/>
       <c r="N18" s="4"/>
       <c r="O18" s="4"/>
-      <c r="P18" s="4"/>
-      <c r="Q18" s="4"/>
+      <c r="P18" s="4">
+        <v>100</v>
+      </c>
+      <c r="Q18" s="4">
+        <v>80</v>
+      </c>
       <c r="R18" s="12"/>
       <c r="S18" s="11">
         <v>1200</v>

</xml_diff>

<commit_message>
Update inventory data 2026-08-31 09:31
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82A1535E-1E2D-4D35-A177-C5DE44011AA4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E13D083B-FDC6-4E41-9B1F-7E163F14511F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2475" yWindow="810" windowWidth="25005" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -990,6 +990,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="8" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{76AA3045-8509-1CC6-4741-1F2A0CDE6A1B}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9324975"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1425,12 +1479,8 @@
       <c r="E5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="4">
-        <v>150</v>
-      </c>
-      <c r="G5" s="4">
-        <v>100</v>
-      </c>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
       <c r="H5" s="4"/>
       <c r="I5" s="4"/>
       <c r="J5" s="4">

</xml_diff>

<commit_message>
Update inventory data 2026-09-10 13:26
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E13D083B-FDC6-4E41-9B1F-7E163F14511F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC654D3E-B755-4A02-AC8D-53F37F9BA0AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2475" yWindow="810" windowWidth="25005" windowHeight="14790" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1335" yWindow="375" windowWidth="22785" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="99">
   <si>
     <t>分類</t>
   </si>
@@ -362,6 +362,17 @@
   </si>
   <si>
     <t>8/17採購617卷，預計九月底完成</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>9/10採購120卷，預計9/17到貨，Sally預約80卷</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>9/10採購40卷，預計9/17到貨</t>
+  </si>
+  <si>
+    <t>9/10採購40卷，預計9/17到貨</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -470,7 +481,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -480,9 +491,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -505,6 +513,15 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1044,6 +1061,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="9" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{46902F40-DF8A-CF61-4AF5-969B2C85360A}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="9525000" cy="9324975"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1277,12 +1348,9 @@
     <col min="3" max="3" width="30.85546875" customWidth="1"/>
     <col min="4" max="4" width="4.42578125" customWidth="1"/>
     <col min="5" max="5" width="6.7109375" customWidth="1"/>
-    <col min="6" max="13" width="17.7109375" customWidth="1"/>
-    <col min="14" max="14" width="9.28515625" customWidth="1"/>
-    <col min="15" max="15" width="8" customWidth="1"/>
-    <col min="16" max="17" width="22" customWidth="1"/>
+    <col min="6" max="17" width="11.42578125" style="14" customWidth="1"/>
     <col min="18" max="18" width="28" customWidth="1"/>
-    <col min="19" max="19" width="14" style="10" customWidth="1"/>
+    <col min="19" max="19" width="14" style="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
@@ -1301,46 +1369,46 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="12" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" s="12" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="R1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="10" t="s">
+      <c r="S1" s="9" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1360,32 +1428,32 @@
       <c r="E2" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F2" s="4"/>
-      <c r="G2" s="4"/>
-      <c r="H2" s="4">
+      <c r="F2" s="13"/>
+      <c r="G2" s="13"/>
+      <c r="H2" s="13">
         <v>100</v>
       </c>
-      <c r="I2" s="4">
+      <c r="I2" s="13">
         <v>60</v>
       </c>
-      <c r="J2" s="4"/>
-      <c r="K2" s="4"/>
-      <c r="L2" s="4"/>
-      <c r="M2" s="4"/>
-      <c r="N2" s="4"/>
-      <c r="O2" s="4"/>
-      <c r="P2" s="4">
+      <c r="J2" s="13"/>
+      <c r="K2" s="13"/>
+      <c r="L2" s="13"/>
+      <c r="M2" s="13"/>
+      <c r="N2" s="13"/>
+      <c r="O2" s="13"/>
+      <c r="P2" s="13">
         <v>200</v>
       </c>
-      <c r="Q2" s="4">
+      <c r="Q2" s="13">
         <v>150</v>
       </c>
-      <c r="R2" s="12"/>
-      <c r="S2" s="11">
+      <c r="R2" s="11"/>
+      <c r="S2" s="10">
         <v>600</v>
       </c>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>18</v>
       </c>
@@ -1401,28 +1469,30 @@
       <c r="E3" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F3" s="4"/>
-      <c r="G3" s="4"/>
-      <c r="H3" s="4"/>
-      <c r="I3" s="4"/>
-      <c r="J3" s="4">
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+      <c r="I3" s="13"/>
+      <c r="J3" s="13">
         <v>40</v>
       </c>
-      <c r="K3" s="4">
+      <c r="K3" s="13">
         <v>25</v>
       </c>
-      <c r="L3" s="4"/>
-      <c r="M3" s="4"/>
-      <c r="N3" s="4"/>
-      <c r="O3" s="4"/>
-      <c r="P3" s="4">
+      <c r="L3" s="13"/>
+      <c r="M3" s="13"/>
+      <c r="N3" s="13"/>
+      <c r="O3" s="13"/>
+      <c r="P3" s="13">
         <v>60</v>
       </c>
-      <c r="Q3" s="4">
+      <c r="Q3" s="13">
         <v>40</v>
       </c>
-      <c r="R3" s="9"/>
-      <c r="S3" s="11">
+      <c r="R3" s="11" t="s">
+        <v>96</v>
+      </c>
+      <c r="S3" s="10">
         <v>900</v>
       </c>
     </row>
@@ -1442,24 +1512,24 @@
       <c r="E4" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F4" s="4">
+      <c r="F4" s="13">
         <v>100</v>
       </c>
-      <c r="G4" s="4">
+      <c r="G4" s="13">
         <v>60</v>
       </c>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="4"/>
-      <c r="O4" s="4"/>
-      <c r="P4" s="4"/>
-      <c r="Q4" s="4"/>
-      <c r="R4" s="9"/>
-      <c r="S4" s="11">
+      <c r="H4" s="13"/>
+      <c r="I4" s="13"/>
+      <c r="J4" s="13"/>
+      <c r="K4" s="13"/>
+      <c r="L4" s="13"/>
+      <c r="M4" s="13"/>
+      <c r="N4" s="13"/>
+      <c r="O4" s="13"/>
+      <c r="P4" s="13"/>
+      <c r="Q4" s="13"/>
+      <c r="R4" s="8"/>
+      <c r="S4" s="10">
         <v>540</v>
       </c>
     </row>
@@ -1479,24 +1549,24 @@
       <c r="E5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4">
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
+      <c r="H5" s="13"/>
+      <c r="I5" s="13"/>
+      <c r="J5" s="13">
         <v>100</v>
       </c>
-      <c r="K5" s="4">
+      <c r="K5" s="13">
         <v>60</v>
       </c>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
-      <c r="P5" s="4"/>
-      <c r="Q5" s="4"/>
-      <c r="R5" s="12"/>
-      <c r="S5" s="11">
+      <c r="L5" s="13"/>
+      <c r="M5" s="13"/>
+      <c r="N5" s="13"/>
+      <c r="O5" s="13"/>
+      <c r="P5" s="13"/>
+      <c r="Q5" s="13"/>
+      <c r="R5" s="11"/>
+      <c r="S5" s="10">
         <v>600</v>
       </c>
     </row>
@@ -1516,24 +1586,26 @@
       <c r="E6" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F6" s="4"/>
-      <c r="G6" s="4"/>
-      <c r="H6" s="4"/>
-      <c r="I6" s="4"/>
-      <c r="J6" s="4">
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="13"/>
+      <c r="I6" s="13"/>
+      <c r="J6" s="13">
         <v>40</v>
       </c>
-      <c r="K6" s="4">
+      <c r="K6" s="13">
         <v>24</v>
       </c>
-      <c r="L6" s="4"/>
-      <c r="M6" s="4"/>
-      <c r="N6" s="4"/>
-      <c r="O6" s="4"/>
-      <c r="P6" s="4"/>
-      <c r="Q6" s="4"/>
-      <c r="R6" s="9"/>
-      <c r="S6" s="11">
+      <c r="L6" s="13"/>
+      <c r="M6" s="13"/>
+      <c r="N6" s="13"/>
+      <c r="O6" s="13"/>
+      <c r="P6" s="13"/>
+      <c r="Q6" s="13"/>
+      <c r="R6" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="S6" s="10">
         <v>960</v>
       </c>
     </row>
@@ -1553,24 +1625,24 @@
       <c r="E7" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
-      <c r="H7" s="4"/>
-      <c r="I7" s="4"/>
-      <c r="J7" s="4">
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="13"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="13">
         <v>40</v>
       </c>
-      <c r="K7" s="4">
+      <c r="K7" s="13">
         <v>24</v>
       </c>
-      <c r="L7" s="4"/>
-      <c r="M7" s="4"/>
-      <c r="N7" s="4"/>
-      <c r="O7" s="4"/>
-      <c r="P7" s="4"/>
-      <c r="Q7" s="4"/>
-      <c r="R7" s="9"/>
-      <c r="S7" s="11">
+      <c r="L7" s="13"/>
+      <c r="M7" s="13"/>
+      <c r="N7" s="13"/>
+      <c r="O7" s="13"/>
+      <c r="P7" s="13"/>
+      <c r="Q7" s="13"/>
+      <c r="R7" s="8"/>
+      <c r="S7" s="10">
         <v>1200</v>
       </c>
     </row>
@@ -1590,28 +1662,28 @@
       <c r="E8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
-      <c r="H8" s="4"/>
-      <c r="I8" s="4"/>
-      <c r="J8" s="4">
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
+      <c r="H8" s="13"/>
+      <c r="I8" s="13"/>
+      <c r="J8" s="13">
         <v>50</v>
       </c>
-      <c r="K8" s="4">
+      <c r="K8" s="13">
         <v>30</v>
       </c>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
-      <c r="N8" s="4"/>
-      <c r="O8" s="4"/>
-      <c r="P8" s="4">
+      <c r="L8" s="13"/>
+      <c r="M8" s="13"/>
+      <c r="N8" s="13"/>
+      <c r="O8" s="13"/>
+      <c r="P8" s="13">
         <v>120</v>
       </c>
-      <c r="Q8" s="4">
+      <c r="Q8" s="13">
         <v>80</v>
       </c>
-      <c r="R8" s="9"/>
-      <c r="S8" s="11">
+      <c r="R8" s="8"/>
+      <c r="S8" s="10">
         <v>600</v>
       </c>
     </row>
@@ -1631,24 +1703,26 @@
       <c r="E9" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F9" s="4"/>
-      <c r="G9" s="4"/>
-      <c r="H9" s="4"/>
-      <c r="I9" s="4"/>
-      <c r="J9" s="4">
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="13"/>
+      <c r="I9" s="13"/>
+      <c r="J9" s="13">
         <v>40</v>
       </c>
-      <c r="K9" s="4">
+      <c r="K9" s="13">
         <v>20</v>
       </c>
-      <c r="L9" s="4"/>
-      <c r="M9" s="4"/>
-      <c r="N9" s="4"/>
-      <c r="O9" s="4"/>
-      <c r="P9" s="4"/>
-      <c r="Q9" s="4"/>
-      <c r="R9" s="9"/>
-      <c r="S9" s="11">
+      <c r="L9" s="13"/>
+      <c r="M9" s="13"/>
+      <c r="N9" s="13"/>
+      <c r="O9" s="13"/>
+      <c r="P9" s="13"/>
+      <c r="Q9" s="13"/>
+      <c r="R9" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="S9" s="10">
         <v>960</v>
       </c>
     </row>
@@ -1668,24 +1742,26 @@
       <c r="E10" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F10" s="4"/>
-      <c r="G10" s="4"/>
-      <c r="H10" s="4"/>
-      <c r="I10" s="4"/>
-      <c r="J10" s="4">
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="13"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="13">
         <v>40</v>
       </c>
-      <c r="K10" s="4">
+      <c r="K10" s="13">
         <v>20</v>
       </c>
-      <c r="L10" s="4"/>
-      <c r="M10" s="4"/>
-      <c r="N10" s="4"/>
-      <c r="O10" s="4"/>
-      <c r="P10" s="4"/>
-      <c r="Q10" s="4"/>
-      <c r="R10" s="9"/>
-      <c r="S10" s="11">
+      <c r="L10" s="13"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="13"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="13"/>
+      <c r="Q10" s="13"/>
+      <c r="R10" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="S10" s="10">
         <v>1200</v>
       </c>
     </row>
@@ -1705,30 +1781,30 @@
       <c r="E11" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
-      <c r="H11" s="4"/>
-      <c r="I11" s="4"/>
-      <c r="J11" s="4">
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="13"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="13">
         <v>120</v>
       </c>
-      <c r="K11" s="4">
+      <c r="K11" s="13">
         <v>60</v>
       </c>
-      <c r="L11" s="4"/>
-      <c r="M11" s="4"/>
-      <c r="N11" s="4"/>
-      <c r="O11" s="4"/>
-      <c r="P11" s="4">
+      <c r="L11" s="13"/>
+      <c r="M11" s="13"/>
+      <c r="N11" s="13"/>
+      <c r="O11" s="13"/>
+      <c r="P11" s="13">
         <v>150</v>
       </c>
-      <c r="Q11" s="4">
+      <c r="Q11" s="13">
         <v>120</v>
       </c>
-      <c r="R11" s="12" t="s">
+      <c r="R11" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="S11" s="11">
+      <c r="S11" s="10">
         <v>990</v>
       </c>
     </row>
@@ -1748,24 +1824,24 @@
       <c r="E12" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
-      <c r="H12" s="4"/>
-      <c r="I12" s="4"/>
-      <c r="J12" s="4">
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13">
         <v>40</v>
       </c>
-      <c r="K12" s="4">
+      <c r="K12" s="13">
         <v>30</v>
       </c>
-      <c r="L12" s="4"/>
-      <c r="M12" s="4"/>
-      <c r="N12" s="4"/>
-      <c r="O12" s="4"/>
-      <c r="P12" s="4"/>
-      <c r="Q12" s="4"/>
-      <c r="R12" s="9"/>
-      <c r="S12" s="11">
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="13"/>
+      <c r="Q12" s="13"/>
+      <c r="R12" s="8"/>
+      <c r="S12" s="10">
         <v>1400</v>
       </c>
     </row>
@@ -1785,22 +1861,22 @@
       <c r="E13" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-      <c r="J13" s="4"/>
-      <c r="K13" s="4">
+      <c r="F13" s="13"/>
+      <c r="G13" s="13"/>
+      <c r="H13" s="13"/>
+      <c r="I13" s="13"/>
+      <c r="J13" s="13"/>
+      <c r="K13" s="13">
         <v>10</v>
       </c>
-      <c r="L13" s="4"/>
-      <c r="M13" s="4"/>
-      <c r="N13" s="4"/>
-      <c r="O13" s="4"/>
-      <c r="P13" s="4"/>
-      <c r="Q13" s="4"/>
-      <c r="R13" s="9"/>
-      <c r="S13" s="11">
+      <c r="L13" s="13"/>
+      <c r="M13" s="13"/>
+      <c r="N13" s="13"/>
+      <c r="O13" s="13"/>
+      <c r="P13" s="13"/>
+      <c r="Q13" s="13"/>
+      <c r="R13" s="8"/>
+      <c r="S13" s="10">
         <v>950</v>
       </c>
     </row>
@@ -1820,24 +1896,24 @@
       <c r="E14" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
-      <c r="I14" s="4"/>
-      <c r="J14" s="4">
+      <c r="F14" s="13"/>
+      <c r="G14" s="13"/>
+      <c r="H14" s="13"/>
+      <c r="I14" s="13"/>
+      <c r="J14" s="13">
         <v>100</v>
       </c>
-      <c r="K14" s="4">
+      <c r="K14" s="13">
         <v>60</v>
       </c>
-      <c r="L14" s="4"/>
-      <c r="M14" s="4"/>
-      <c r="N14" s="4"/>
-      <c r="O14" s="4"/>
-      <c r="P14" s="4"/>
-      <c r="Q14" s="4"/>
-      <c r="R14" s="9"/>
-      <c r="S14" s="11">
+      <c r="L14" s="13"/>
+      <c r="M14" s="13"/>
+      <c r="N14" s="13"/>
+      <c r="O14" s="13"/>
+      <c r="P14" s="13"/>
+      <c r="Q14" s="13"/>
+      <c r="R14" s="8"/>
+      <c r="S14" s="10">
         <v>600</v>
       </c>
     </row>
@@ -1857,24 +1933,24 @@
       <c r="E15" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
-      <c r="I15" s="4"/>
-      <c r="J15" s="4">
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="13"/>
+      <c r="J15" s="13">
         <v>30</v>
       </c>
-      <c r="K15" s="4">
+      <c r="K15" s="13">
         <v>10</v>
       </c>
-      <c r="L15" s="4"/>
-      <c r="M15" s="4"/>
-      <c r="N15" s="4"/>
-      <c r="O15" s="4"/>
-      <c r="P15" s="4"/>
-      <c r="Q15" s="4"/>
-      <c r="R15" s="9"/>
-      <c r="S15" s="11">
+      <c r="L15" s="13"/>
+      <c r="M15" s="13"/>
+      <c r="N15" s="13"/>
+      <c r="O15" s="13"/>
+      <c r="P15" s="13"/>
+      <c r="Q15" s="13"/>
+      <c r="R15" s="8"/>
+      <c r="S15" s="10">
         <v>600</v>
       </c>
     </row>
@@ -1894,24 +1970,24 @@
       <c r="E16" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-      <c r="J16" s="4">
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
+      <c r="I16" s="13"/>
+      <c r="J16" s="13">
         <v>40</v>
       </c>
-      <c r="K16" s="4">
+      <c r="K16" s="13">
         <v>24</v>
       </c>
-      <c r="L16" s="4"/>
-      <c r="M16" s="4"/>
-      <c r="N16" s="4"/>
-      <c r="O16" s="4"/>
-      <c r="P16" s="4"/>
-      <c r="Q16" s="4"/>
-      <c r="R16" s="9"/>
-      <c r="S16" s="11">
+      <c r="L16" s="13"/>
+      <c r="M16" s="13"/>
+      <c r="N16" s="13"/>
+      <c r="O16" s="13"/>
+      <c r="P16" s="13"/>
+      <c r="Q16" s="13"/>
+      <c r="R16" s="8"/>
+      <c r="S16" s="10">
         <v>1400</v>
       </c>
     </row>
@@ -1931,24 +2007,24 @@
       <c r="E17" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F17" s="4"/>
-      <c r="G17" s="4"/>
-      <c r="H17" s="4"/>
-      <c r="I17" s="4"/>
-      <c r="J17" s="4"/>
-      <c r="K17" s="4"/>
-      <c r="L17" s="4"/>
-      <c r="M17" s="4"/>
-      <c r="N17" s="4"/>
-      <c r="O17" s="4"/>
-      <c r="P17" s="4">
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+      <c r="I17" s="13"/>
+      <c r="J17" s="13"/>
+      <c r="K17" s="13"/>
+      <c r="L17" s="13"/>
+      <c r="M17" s="13"/>
+      <c r="N17" s="13"/>
+      <c r="O17" s="13"/>
+      <c r="P17" s="13">
         <v>40</v>
       </c>
-      <c r="Q17" s="4">
+      <c r="Q17" s="13">
         <v>20</v>
       </c>
-      <c r="R17" s="9"/>
-      <c r="S17" s="11">
+      <c r="R17" s="8"/>
+      <c r="S17" s="10">
         <v>1200</v>
       </c>
     </row>
@@ -1968,24 +2044,24 @@
       <c r="E18" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F18" s="4"/>
-      <c r="G18" s="4"/>
-      <c r="H18" s="4"/>
-      <c r="I18" s="4"/>
-      <c r="J18" s="4"/>
-      <c r="K18" s="4"/>
-      <c r="L18" s="4"/>
-      <c r="M18" s="4"/>
-      <c r="N18" s="4"/>
-      <c r="O18" s="4"/>
-      <c r="P18" s="4">
+      <c r="F18" s="13"/>
+      <c r="G18" s="13"/>
+      <c r="H18" s="13"/>
+      <c r="I18" s="13"/>
+      <c r="J18" s="13"/>
+      <c r="K18" s="13"/>
+      <c r="L18" s="13"/>
+      <c r="M18" s="13"/>
+      <c r="N18" s="13"/>
+      <c r="O18" s="13"/>
+      <c r="P18" s="13">
         <v>100</v>
       </c>
-      <c r="Q18" s="4">
+      <c r="Q18" s="13">
         <v>80</v>
       </c>
-      <c r="R18" s="12"/>
-      <c r="S18" s="11">
+      <c r="R18" s="11"/>
+      <c r="S18" s="10">
         <v>1200</v>
       </c>
     </row>
@@ -2005,24 +2081,24 @@
       <c r="E19" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F19" s="4"/>
-      <c r="G19" s="4"/>
-      <c r="H19" s="4"/>
-      <c r="I19" s="4"/>
-      <c r="J19" s="4"/>
-      <c r="K19" s="4"/>
-      <c r="L19" s="4"/>
-      <c r="M19" s="4"/>
-      <c r="N19" s="4">
+      <c r="F19" s="13"/>
+      <c r="G19" s="13"/>
+      <c r="H19" s="13"/>
+      <c r="I19" s="13"/>
+      <c r="J19" s="13"/>
+      <c r="K19" s="13"/>
+      <c r="L19" s="13"/>
+      <c r="M19" s="13"/>
+      <c r="N19" s="13">
         <v>100</v>
       </c>
-      <c r="O19" s="4">
+      <c r="O19" s="13">
         <v>80</v>
       </c>
-      <c r="P19" s="4"/>
-      <c r="Q19" s="4"/>
-      <c r="R19" s="9"/>
-      <c r="S19" s="11"/>
+      <c r="P19" s="13"/>
+      <c r="Q19" s="13"/>
+      <c r="R19" s="8"/>
+      <c r="S19" s="10"/>
     </row>
     <row r="20" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
@@ -2040,24 +2116,24 @@
       <c r="E20" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F20" s="4"/>
-      <c r="G20" s="4"/>
-      <c r="H20" s="4"/>
-      <c r="I20" s="4"/>
-      <c r="J20" s="4"/>
-      <c r="K20" s="4"/>
-      <c r="L20" s="4"/>
-      <c r="M20" s="4"/>
-      <c r="N20" s="4"/>
-      <c r="O20" s="4"/>
-      <c r="P20" s="4">
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="13"/>
+      <c r="I20" s="13"/>
+      <c r="J20" s="13"/>
+      <c r="K20" s="13"/>
+      <c r="L20" s="13"/>
+      <c r="M20" s="13"/>
+      <c r="N20" s="13"/>
+      <c r="O20" s="13"/>
+      <c r="P20" s="13">
         <v>20</v>
       </c>
-      <c r="Q20" s="4">
+      <c r="Q20" s="13">
         <v>8</v>
       </c>
-      <c r="R20" s="9"/>
-      <c r="S20" s="11"/>
+      <c r="R20" s="8"/>
+      <c r="S20" s="10"/>
     </row>
     <row r="21" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
@@ -2075,22 +2151,22 @@
       <c r="E21" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F21" s="4"/>
-      <c r="G21" s="4"/>
-      <c r="H21" s="4"/>
-      <c r="I21" s="4"/>
-      <c r="J21" s="4"/>
-      <c r="K21" s="4"/>
-      <c r="L21" s="4"/>
-      <c r="M21" s="4"/>
-      <c r="N21" s="4"/>
-      <c r="O21" s="4"/>
-      <c r="P21" s="4">
+      <c r="F21" s="13"/>
+      <c r="G21" s="13"/>
+      <c r="H21" s="13"/>
+      <c r="I21" s="13"/>
+      <c r="J21" s="13"/>
+      <c r="K21" s="13"/>
+      <c r="L21" s="13"/>
+      <c r="M21" s="13"/>
+      <c r="N21" s="13"/>
+      <c r="O21" s="13"/>
+      <c r="P21" s="13">
         <v>20</v>
       </c>
-      <c r="Q21" s="4"/>
-      <c r="R21" s="9"/>
-      <c r="S21" s="11"/>
+      <c r="Q21" s="13"/>
+      <c r="R21" s="8"/>
+      <c r="S21" s="10"/>
     </row>
     <row r="22" spans="1:19" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
@@ -2108,20 +2184,20 @@
       <c r="E22" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
-      <c r="H22" s="4"/>
-      <c r="I22" s="4"/>
-      <c r="J22" s="4"/>
-      <c r="K22" s="4"/>
-      <c r="L22" s="4"/>
-      <c r="M22" s="4"/>
-      <c r="N22" s="4"/>
-      <c r="O22" s="4"/>
-      <c r="P22" s="4"/>
-      <c r="Q22" s="4"/>
-      <c r="R22" s="9"/>
-      <c r="S22" s="11">
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+      <c r="I22" s="13"/>
+      <c r="J22" s="13"/>
+      <c r="K22" s="13"/>
+      <c r="L22" s="13"/>
+      <c r="M22" s="13"/>
+      <c r="N22" s="13"/>
+      <c r="O22" s="13"/>
+      <c r="P22" s="13"/>
+      <c r="Q22" s="13"/>
+      <c r="R22" s="8"/>
+      <c r="S22" s="10">
         <v>900</v>
       </c>
     </row>
@@ -2141,20 +2217,20 @@
       <c r="E23" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F23" s="4"/>
-      <c r="G23" s="4"/>
-      <c r="H23" s="4"/>
-      <c r="I23" s="4"/>
-      <c r="J23" s="4"/>
-      <c r="K23" s="4"/>
-      <c r="L23" s="4"/>
-      <c r="M23" s="4"/>
-      <c r="N23" s="4"/>
-      <c r="O23" s="4"/>
-      <c r="P23" s="4"/>
-      <c r="Q23" s="4"/>
-      <c r="R23" s="9"/>
-      <c r="S23" s="11">
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13"/>
+      <c r="K23" s="13"/>
+      <c r="L23" s="13"/>
+      <c r="M23" s="13"/>
+      <c r="N23" s="13"/>
+      <c r="O23" s="13"/>
+      <c r="P23" s="13"/>
+      <c r="Q23" s="13"/>
+      <c r="R23" s="8"/>
+      <c r="S23" s="10">
         <v>1400</v>
       </c>
     </row>
@@ -2174,20 +2250,20 @@
       <c r="E24" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F24" s="4"/>
-      <c r="G24" s="4"/>
-      <c r="H24" s="4"/>
-      <c r="I24" s="4"/>
-      <c r="J24" s="4"/>
-      <c r="K24" s="4"/>
-      <c r="L24" s="4"/>
-      <c r="M24" s="4"/>
-      <c r="N24" s="4"/>
-      <c r="O24" s="4"/>
-      <c r="P24" s="4"/>
-      <c r="Q24" s="4"/>
-      <c r="R24" s="9"/>
-      <c r="S24" s="11"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13"/>
+      <c r="K24" s="13"/>
+      <c r="L24" s="13"/>
+      <c r="M24" s="13"/>
+      <c r="N24" s="13"/>
+      <c r="O24" s="13"/>
+      <c r="P24" s="13"/>
+      <c r="Q24" s="13"/>
+      <c r="R24" s="8"/>
+      <c r="S24" s="10"/>
     </row>
     <row r="25" spans="1:19" ht="47.25" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
@@ -2205,24 +2281,24 @@
       <c r="E25" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
-      <c r="H25" s="4"/>
-      <c r="I25" s="4"/>
-      <c r="J25" s="4"/>
-      <c r="K25" s="4"/>
-      <c r="L25" s="4"/>
-      <c r="M25" s="4"/>
-      <c r="N25" s="4"/>
-      <c r="O25" s="4"/>
-      <c r="P25" s="4">
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+      <c r="H25" s="13"/>
+      <c r="I25" s="13"/>
+      <c r="J25" s="13"/>
+      <c r="K25" s="13"/>
+      <c r="L25" s="13"/>
+      <c r="M25" s="13"/>
+      <c r="N25" s="13"/>
+      <c r="O25" s="13"/>
+      <c r="P25" s="13">
         <v>80</v>
       </c>
-      <c r="Q25" s="4">
+      <c r="Q25" s="13">
         <v>50</v>
       </c>
-      <c r="R25" s="9"/>
-      <c r="S25" s="11"/>
+      <c r="R25" s="8"/>
+      <c r="S25" s="10"/>
     </row>
     <row r="26" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
@@ -2240,24 +2316,24 @@
       <c r="E26" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
-      <c r="H26" s="4"/>
-      <c r="I26" s="4"/>
-      <c r="J26" s="4">
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
+      <c r="I26" s="13"/>
+      <c r="J26" s="13">
         <v>60</v>
       </c>
-      <c r="K26" s="4">
+      <c r="K26" s="13">
         <v>40</v>
       </c>
-      <c r="L26" s="4"/>
-      <c r="M26" s="4"/>
-      <c r="N26" s="4"/>
-      <c r="O26" s="4"/>
-      <c r="P26" s="4"/>
-      <c r="Q26" s="4"/>
-      <c r="R26" s="9"/>
-      <c r="S26" s="11">
+      <c r="L26" s="13"/>
+      <c r="M26" s="13"/>
+      <c r="N26" s="13"/>
+      <c r="O26" s="13"/>
+      <c r="P26" s="13"/>
+      <c r="Q26" s="13"/>
+      <c r="R26" s="8"/>
+      <c r="S26" s="10">
         <v>600</v>
       </c>
     </row>
@@ -2277,20 +2353,20 @@
       <c r="E27" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F27" s="4"/>
-      <c r="G27" s="4"/>
-      <c r="H27" s="4"/>
-      <c r="I27" s="4"/>
-      <c r="J27" s="4"/>
-      <c r="K27" s="4"/>
-      <c r="L27" s="4"/>
-      <c r="M27" s="4"/>
-      <c r="N27" s="4"/>
-      <c r="O27" s="4"/>
-      <c r="P27" s="4"/>
-      <c r="Q27" s="4"/>
-      <c r="R27" s="9"/>
-      <c r="S27" s="11">
+      <c r="F27" s="13"/>
+      <c r="G27" s="13"/>
+      <c r="H27" s="13"/>
+      <c r="I27" s="13"/>
+      <c r="J27" s="13"/>
+      <c r="K27" s="13"/>
+      <c r="L27" s="13"/>
+      <c r="M27" s="13"/>
+      <c r="N27" s="13"/>
+      <c r="O27" s="13"/>
+      <c r="P27" s="13"/>
+      <c r="Q27" s="13"/>
+      <c r="R27" s="8"/>
+      <c r="S27" s="10">
         <v>600</v>
       </c>
     </row>
@@ -2310,20 +2386,20 @@
       <c r="E28" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
-      <c r="H28" s="4"/>
-      <c r="I28" s="4"/>
-      <c r="J28" s="4"/>
-      <c r="K28" s="4"/>
-      <c r="L28" s="4"/>
-      <c r="M28" s="4"/>
-      <c r="N28" s="4"/>
-      <c r="O28" s="4"/>
-      <c r="P28" s="4"/>
-      <c r="Q28" s="4"/>
-      <c r="R28" s="9"/>
-      <c r="S28" s="11">
+      <c r="F28" s="13"/>
+      <c r="G28" s="13"/>
+      <c r="H28" s="13"/>
+      <c r="I28" s="13"/>
+      <c r="J28" s="13"/>
+      <c r="K28" s="13"/>
+      <c r="L28" s="13"/>
+      <c r="M28" s="13"/>
+      <c r="N28" s="13"/>
+      <c r="O28" s="13"/>
+      <c r="P28" s="13"/>
+      <c r="Q28" s="13"/>
+      <c r="R28" s="8"/>
+      <c r="S28" s="10">
         <v>600</v>
       </c>
     </row>
@@ -2343,20 +2419,20 @@
       <c r="E29" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F29" s="4"/>
-      <c r="G29" s="4"/>
-      <c r="H29" s="4"/>
-      <c r="I29" s="4"/>
-      <c r="J29" s="4"/>
-      <c r="K29" s="4"/>
-      <c r="L29" s="4"/>
-      <c r="M29" s="4"/>
-      <c r="N29" s="4"/>
-      <c r="O29" s="4"/>
-      <c r="P29" s="4"/>
-      <c r="Q29" s="4"/>
-      <c r="R29" s="9"/>
-      <c r="S29" s="11">
+      <c r="F29" s="13"/>
+      <c r="G29" s="13"/>
+      <c r="H29" s="13"/>
+      <c r="I29" s="13"/>
+      <c r="J29" s="13"/>
+      <c r="K29" s="13"/>
+      <c r="L29" s="13"/>
+      <c r="M29" s="13"/>
+      <c r="N29" s="13"/>
+      <c r="O29" s="13"/>
+      <c r="P29" s="13"/>
+      <c r="Q29" s="13"/>
+      <c r="R29" s="8"/>
+      <c r="S29" s="10">
         <v>600</v>
       </c>
     </row>
@@ -2376,24 +2452,24 @@
       <c r="E30" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F30" s="4"/>
-      <c r="G30" s="4"/>
-      <c r="H30" s="4"/>
-      <c r="I30" s="4"/>
-      <c r="J30" s="4">
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
+      <c r="H30" s="13"/>
+      <c r="I30" s="13"/>
+      <c r="J30" s="13">
         <v>60</v>
       </c>
-      <c r="K30" s="4">
+      <c r="K30" s="13">
         <v>40</v>
       </c>
-      <c r="L30" s="4"/>
-      <c r="M30" s="4"/>
-      <c r="N30" s="4"/>
-      <c r="O30" s="4"/>
-      <c r="P30" s="4"/>
-      <c r="Q30" s="4"/>
-      <c r="R30" s="9"/>
-      <c r="S30" s="11">
+      <c r="L30" s="13"/>
+      <c r="M30" s="13"/>
+      <c r="N30" s="13"/>
+      <c r="O30" s="13"/>
+      <c r="P30" s="13"/>
+      <c r="Q30" s="13"/>
+      <c r="R30" s="8"/>
+      <c r="S30" s="10">
         <v>600</v>
       </c>
     </row>
@@ -2413,24 +2489,24 @@
       <c r="E31" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F31" s="4"/>
-      <c r="G31" s="4"/>
-      <c r="H31" s="4"/>
-      <c r="I31" s="4"/>
-      <c r="J31" s="4">
+      <c r="F31" s="13"/>
+      <c r="G31" s="13"/>
+      <c r="H31" s="13"/>
+      <c r="I31" s="13"/>
+      <c r="J31" s="13">
         <v>60</v>
       </c>
-      <c r="K31" s="4">
+      <c r="K31" s="13">
         <v>40</v>
       </c>
-      <c r="L31" s="4"/>
-      <c r="M31" s="4"/>
-      <c r="N31" s="4"/>
-      <c r="O31" s="4"/>
-      <c r="P31" s="4"/>
-      <c r="Q31" s="4"/>
-      <c r="R31" s="9"/>
-      <c r="S31" s="11">
+      <c r="L31" s="13"/>
+      <c r="M31" s="13"/>
+      <c r="N31" s="13"/>
+      <c r="O31" s="13"/>
+      <c r="P31" s="13"/>
+      <c r="Q31" s="13"/>
+      <c r="R31" s="8"/>
+      <c r="S31" s="10">
         <v>900</v>
       </c>
     </row>
@@ -2450,20 +2526,20 @@
       <c r="E32" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F32" s="4"/>
-      <c r="G32" s="4"/>
-      <c r="H32" s="4"/>
-      <c r="I32" s="4"/>
-      <c r="J32" s="4"/>
-      <c r="K32" s="4"/>
-      <c r="L32" s="4"/>
-      <c r="M32" s="4"/>
-      <c r="N32" s="4"/>
-      <c r="O32" s="4"/>
-      <c r="P32" s="4"/>
-      <c r="Q32" s="4"/>
-      <c r="R32" s="9"/>
-      <c r="S32" s="11">
+      <c r="F32" s="13"/>
+      <c r="G32" s="13"/>
+      <c r="H32" s="13"/>
+      <c r="I32" s="13"/>
+      <c r="J32" s="13"/>
+      <c r="K32" s="13"/>
+      <c r="L32" s="13"/>
+      <c r="M32" s="13"/>
+      <c r="N32" s="13"/>
+      <c r="O32" s="13"/>
+      <c r="P32" s="13"/>
+      <c r="Q32" s="13"/>
+      <c r="R32" s="8"/>
+      <c r="S32" s="10">
         <v>900</v>
       </c>
     </row>
@@ -2483,20 +2559,20 @@
       <c r="E33" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F33" s="4"/>
-      <c r="G33" s="4"/>
-      <c r="H33" s="4"/>
-      <c r="I33" s="4"/>
-      <c r="J33" s="4"/>
-      <c r="K33" s="4"/>
-      <c r="L33" s="4"/>
-      <c r="M33" s="4"/>
-      <c r="N33" s="4"/>
-      <c r="O33" s="4"/>
-      <c r="P33" s="4"/>
-      <c r="Q33" s="4"/>
-      <c r="R33" s="9"/>
-      <c r="S33" s="11">
+      <c r="F33" s="13"/>
+      <c r="G33" s="13"/>
+      <c r="H33" s="13"/>
+      <c r="I33" s="13"/>
+      <c r="J33" s="13"/>
+      <c r="K33" s="13"/>
+      <c r="L33" s="13"/>
+      <c r="M33" s="13"/>
+      <c r="N33" s="13"/>
+      <c r="O33" s="13"/>
+      <c r="P33" s="13"/>
+      <c r="Q33" s="13"/>
+      <c r="R33" s="8"/>
+      <c r="S33" s="10">
         <v>900</v>
       </c>
     </row>
@@ -2516,20 +2592,20 @@
       <c r="E34" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="F34" s="4"/>
-      <c r="G34" s="4"/>
-      <c r="H34" s="4"/>
-      <c r="I34" s="4"/>
-      <c r="J34" s="4"/>
-      <c r="K34" s="4"/>
-      <c r="L34" s="4"/>
-      <c r="M34" s="4"/>
-      <c r="N34" s="4"/>
-      <c r="O34" s="4"/>
-      <c r="P34" s="4"/>
-      <c r="Q34" s="4"/>
-      <c r="R34" s="9"/>
-      <c r="S34" s="11">
+      <c r="F34" s="13"/>
+      <c r="G34" s="13"/>
+      <c r="H34" s="13"/>
+      <c r="I34" s="13"/>
+      <c r="J34" s="13"/>
+      <c r="K34" s="13"/>
+      <c r="L34" s="13"/>
+      <c r="M34" s="13"/>
+      <c r="N34" s="13"/>
+      <c r="O34" s="13"/>
+      <c r="P34" s="13"/>
+      <c r="Q34" s="13"/>
+      <c r="R34" s="8"/>
+      <c r="S34" s="10">
         <v>900</v>
       </c>
     </row>
@@ -2624,74 +2700,74 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>71</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>73</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A8" s="6" t="s">
+      <c r="A8" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="B8" s="6" t="s">
+      <c r="B8" s="5" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A9" s="6" t="s">
+      <c r="A9" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="B9" s="6" t="s">
+      <c r="B9" s="5" t="s">
         <v>78</v>
       </c>
     </row>
@@ -2699,7 +2775,7 @@
       <c r="A10" t="s">
         <v>93</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>94</v>
       </c>
     </row>
@@ -2719,58 +2795,58 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>79</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="4" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" s="6" t="s">
+      <c r="A2" s="5" t="s">
         <v>81</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="5" t="s">
         <v>85</v>
       </c>
-      <c r="B4" s="6" t="s">
+      <c r="B4" s="5" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="B5" s="5" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" s="6" t="s">
+      <c r="A6" s="5" t="s">
         <v>89</v>
       </c>
-      <c r="B6" s="6" t="s">
+      <c r="B6" s="5" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" s="6" t="s">
+      <c r="A7" s="5" t="s">
         <v>91</v>
       </c>
-      <c r="B7" s="6" t="s">
+      <c r="B7" s="5" t="s">
         <v>92</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update inventory data 2026-09-10 14:12
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC654D3E-B755-4A02-AC8D-53F37F9BA0AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30C66014-8E51-45DB-A885-BD32A090B4AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1335" yWindow="375" windowWidth="22785" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="101">
   <si>
     <t>分類</t>
   </si>
@@ -373,6 +373,14 @@
   </si>
   <si>
     <t>9/10採購40卷，預計9/17到貨</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>9/10採購411卷，交期未知</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>9/10採購206卷，交期未知</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1115,6 +1123,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="10" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{55FD13FA-8D8D-07BA-4D9A-63949F3F06DE}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7848600" cy="9525000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1912,7 +1974,9 @@
       <c r="O14" s="13"/>
       <c r="P14" s="13"/>
       <c r="Q14" s="13"/>
-      <c r="R14" s="8"/>
+      <c r="R14" s="11" t="s">
+        <v>99</v>
+      </c>
       <c r="S14" s="10">
         <v>600</v>
       </c>
@@ -1949,7 +2013,9 @@
       <c r="O15" s="13"/>
       <c r="P15" s="13"/>
       <c r="Q15" s="13"/>
-      <c r="R15" s="8"/>
+      <c r="R15" s="11" t="s">
+        <v>100</v>
+      </c>
       <c r="S15" s="10">
         <v>600</v>
       </c>

</xml_diff>

<commit_message>
Update inventory data 2026-09-11 09:14
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30C66014-8E51-45DB-A885-BD32A090B4AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{174B7E48-62A7-4F4D-9409-4A4888A1C7AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1335" yWindow="375" windowWidth="22785" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="750" yWindow="420" windowWidth="22785" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="採購提醒設定" sheetId="1" r:id="rId1"/>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="102">
   <si>
     <t>分類</t>
   </si>
@@ -381,6 +381,10 @@
   </si>
   <si>
     <t>9/10採購206卷，交期未知</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>9/10採購124卷，交期未知</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1177,6 +1181,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="11" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{707227BE-6FC7-C685-BED6-D08E38E65FF3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7848600" cy="9525000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -1937,7 +1995,9 @@
       <c r="O13" s="13"/>
       <c r="P13" s="13"/>
       <c r="Q13" s="13"/>
-      <c r="R13" s="8"/>
+      <c r="R13" s="11" t="s">
+        <v>101</v>
+      </c>
       <c r="S13" s="10">
         <v>950</v>
       </c>

</xml_diff>

<commit_message>
Update inventory data 2026-09-11 11:53
</commit_message>
<xml_diff>
--- a/data/採購提醒設定.xlsx
+++ b/data/採購提醒設定.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\封王封膜庫存監控\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{174B7E48-62A7-4F4D-9409-4A4888A1C7AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{139ACDA5-A662-4A1A-99B8-45C38D56074B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="750" yWindow="420" windowWidth="22785" windowHeight="15180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="103">
   <si>
     <t>分類</t>
   </si>
@@ -385,6 +385,10 @@
   </si>
   <si>
     <t>9/10採購124卷，交期未知</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>9/11採購103卷，交期未知</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1235,6 +1239,60 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>561975</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="12" name="AutoShape 4">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{FFE056E0-D957-A359-4709-738A42664663}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr>
+          <a:spLocks noChangeArrowheads="1"/>
+        </xdr:cNvSpPr>
+      </xdr:nvSpPr>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="0" y="0"/>
+          <a:ext cx="7848600" cy="9525000"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="0" t="0" r="0" b="0"/>
+          <a:pathLst/>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+          <a:round/>
+          <a:headEnd/>
+          <a:tailEnd/>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 
@@ -2112,7 +2170,9 @@
       <c r="O16" s="13"/>
       <c r="P16" s="13"/>
       <c r="Q16" s="13"/>
-      <c r="R16" s="8"/>
+      <c r="R16" s="11" t="s">
+        <v>102</v>
+      </c>
       <c r="S16" s="10">
         <v>1400</v>
       </c>

</xml_diff>